<commit_message>
fase 2: orcamento de buffet (aba Buffet na planilha + pedidos 7-9)
</commit_message>
<xml_diff>
--- a/planilha/lanchonete-bom-pedaco.xlsx
+++ b/planilha/lanchonete-bom-pedaco.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Vendas" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Sobre" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Buffet" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;R$&quot; #,##0.00"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,6 +43,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="3">
@@ -69,7 +74,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -78,6 +83,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4703,7 +4710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -4758,6 +4765,320 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>A aba Buffet</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>A lanchonete também faz buffet para festas e eventos. A aba Buffet traz os pacotes, os extras e as regras para montar um orçamento.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Buffet Bom Pedaço: pacotes, extras e regras de orçamento</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>DADOS FICTÍCIOS, criados para a imersão IA para empresários. Não representam nenhuma empresa real.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>PACOTES (preço por convidado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Pacote</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>O que inclui</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Preço por convidado (R$)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Coffee break</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mini sanduíches, pão de queijo, bolo, café e suco</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Festa de lanches</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Mini X-Burger, mini X-Salada, batata frita, refrigerante e suco</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Festa completa</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Tudo da Festa de lanches + Smash Duplo feito na chapa na hora + sobremesa</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>EXTRAS (preço por convidado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Extra</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>O que é</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Preço por convidado (R$)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Mesa de doces</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Brigadeiro, beijinho e cajuzinho</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Bolo decorado</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Bolo de 2 andares, sabor à escolha</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Louça e toalhas</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Pratos, talheres, copos de vidro e toalhas de mesa</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>REGRAS DO ORÇAMENTO (aplicar nesta ordem)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Nº</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Regra</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Mínimo de 30 convidados. Com menos de 30, cobra-se como 30.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>2</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Valor do pacote = convidados × preço por convidado do pacote escolhido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>3</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Sábado, domingo ou feriado: +15% sobre o valor do pacote (não vale para os extras).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>A partir de 100 convidados: 10% de desconto sobre o valor do pacote, já com o acréscimo da regra 3 (não vale para os extras).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>5</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Extras = convidados × preço por convidado de cada extra escolhido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>6</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Equipe: 1 atendente para cada 25 convidados, arredondando para cima. R$ 180 por atendente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>7</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Duração padrão: 4 horas de festa. Cada hora a mais custa R$ 300.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>8</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Deslocamento: até 10 km da lanchonete, grátis. Acima disso, R$ 5 por km além dos 10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>9</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Total = pacote + extras + equipe + horas extras + deslocamento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>10</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Sinal de 30% do total para reservar a data. O restante é pago até 3 dias antes da festa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>11</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>O orçamento vale por 7 dias. Festas com menos de 7 dias de antecedência precisam de confirmação do dono.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>